<commit_message>
to rework images and hero
</commit_message>
<xml_diff>
--- a/src/content/content_TEMPLATE.xlsx
+++ b/src/content/content_TEMPLATE.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -609,31 +609,31 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>text</v>
+        <v>languageSwitcher</v>
       </c>
       <c r="C6" t="str">
-        <v>Цей текст відображається як звичайний абзац.</v>
+        <v>UA</v>
       </c>
       <c r="D6" t="str">
-        <v>Этот текст выводится как обычный параграф.</v>
+        <v>RU</v>
       </c>
       <c r="E6" t="str">
-        <v>This text is rendered as a normal paragraph.</v>
+        <v>EN</v>
       </c>
       <c r="F6" t="str">
-        <v>Dieser Text wird als normaler Absatz angezeigt.</v>
+        <v>DE</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>Переключатель языка</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>Переключатель языка</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>Language switcher</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>Sprachumschalter</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -647,19 +647,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>image</v>
+        <v>text</v>
       </c>
       <c r="C7" t="str">
-        <v>images/example.jpg</v>
+        <v>Цей текст відображається як звичайний абзац.</v>
       </c>
       <c r="D7" t="str">
-        <v>images/example.jpg</v>
+        <v>Этот текст выводится как обычный параграф.</v>
       </c>
       <c r="E7" t="str">
-        <v>images/example.jpg</v>
+        <v>This text is rendered as a normal paragraph.</v>
       </c>
       <c r="F7" t="str">
-        <v>images/example.jpg</v>
+        <v>Dieser Text wird als normaler Absatz angezeigt.</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -677,27 +677,27 @@
         <v/>
       </c>
       <c r="L7" t="str">
-        <v>w=600;h=400;resizeMode=contain</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="str">
-        <v>gif</v>
+        <v>image</v>
       </c>
       <c r="C8" t="str">
-        <v>images/animation.gif</v>
+        <v>images/example.jpg</v>
       </c>
       <c r="D8" t="str">
-        <v>images/animation.gif</v>
+        <v>images/example.jpg</v>
       </c>
       <c r="E8" t="str">
-        <v>images/animation.gif</v>
+        <v>images/example.jpg</v>
       </c>
       <c r="F8" t="str">
-        <v>images/animation.gif</v>
+        <v>images/example.jpg</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -715,80 +715,80 @@
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>w=400;h=225;resizeMode=contain</v>
+        <v>w=600;h=400;resizeMode=contain</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="str">
-        <v>card</v>
+        <v>gif</v>
       </c>
       <c r="C9" t="str">
-        <v>Заголовок карточки</v>
+        <v>images/animation.gif</v>
       </c>
       <c r="D9" t="str">
-        <v>Заголовок карточки</v>
+        <v>images/animation.gif</v>
       </c>
       <c r="E9" t="str">
-        <v>Card title</v>
+        <v>images/animation.gif</v>
       </c>
       <c r="F9" t="str">
-        <v>Kartenüberschrift</v>
+        <v>images/animation.gif</v>
       </c>
       <c r="G9" t="str">
-        <v>Опис карточки українською</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>Описание карточки на русском</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>Card description in English</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>Kartenbeschreibung auf Deutsch</v>
+        <v/>
       </c>
       <c r="K9" t="str">
-        <v>/lesson-example</v>
+        <v/>
       </c>
       <c r="L9" t="str">
-        <v/>
+        <v>w=400;h=225;resizeMode=contain</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="str">
-        <v>video</v>
+        <v>card</v>
       </c>
       <c r="C10" t="str">
-        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
+        <v>Заголовок карточки</v>
       </c>
       <c r="D10" t="str">
-        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
+        <v>Заголовок карточки</v>
       </c>
       <c r="E10" t="str">
-        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
+        <v>Card title</v>
       </c>
       <c r="F10" t="str">
-        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
+        <v>Kartenüberschrift</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>Опис карточки українською</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>Описание карточки на русском</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>Card description in English</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>Kartenbeschreibung auf Deutsch</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>/lesson-example</v>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -796,22 +796,22 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="str">
-        <v>link</v>
+        <v>video</v>
       </c>
       <c r="C11" t="str">
-        <v>Детальніше про курс</v>
+        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
       </c>
       <c r="D11" t="str">
-        <v>Подробнее о курсе</v>
+        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
       </c>
       <c r="E11" t="str">
-        <v>Read more about the course</v>
+        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
       </c>
       <c r="F11" t="str">
-        <v>Mehr über den Kurs</v>
+        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
       </c>
       <c r="G11" t="str">
         <v/>
@@ -826,7 +826,7 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>/course</v>
+        <v/>
       </c>
       <c r="L11" t="str">
         <v/>
@@ -834,22 +834,22 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="str">
-        <v>item</v>
+        <v>link</v>
       </c>
       <c r="C12" t="str">
-        <v>Пункт списку UA</v>
+        <v>Детальніше про курс</v>
       </c>
       <c r="D12" t="str">
-        <v>Пункт списка RU</v>
+        <v>Подробнее о курсе</v>
       </c>
       <c r="E12" t="str">
-        <v>List item EN</v>
+        <v>Read more about the course</v>
       </c>
       <c r="F12" t="str">
-        <v>Listenelement DE</v>
+        <v>Mehr über den Kurs</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -864,7 +864,7 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>/course</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -872,45 +872,83 @@
     </row>
     <row r="13">
       <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>item</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Пункт списку UA</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Пункт списка RU</v>
+      </c>
+      <c r="E13" t="str">
+        <v>List item EN</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Listenelement DE</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
         <v>12</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B14" t="str">
         <v>navigationButtons</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C14" t="str">
         <v>Наступний урок</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D14" t="str">
         <v>Следующий урок</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E14" t="str">
         <v>Next lesson</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F14" t="str">
         <v>Nächste Lektion</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13" t="str">
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
         <v>/next-page</v>
       </c>
-      <c r="L13" t="str">
+      <c r="L14" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>